<commit_message>
Add Riyadh operating expenses before 30-7-2025
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/المصاريف_التشغيلية_مزرعة_الرياض_2026.xlsx
+++ b/المصاريف_التشغيلية_مزرعة_الرياض_2026.xlsx
@@ -8,16 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="الملخص" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="أوامر الشراء" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="العهد - تفصيل المصروفات" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="العهد - ملخص" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="مصروفات 2025 - تفصيل" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="مصروفات 2025 - ملخص" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="مصروفات قبل 30.7.2025" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="أوامر الشراء" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="العهد - تفصيل المصروفات" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="العهد - ملخص" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="مصروفات 2025 - تفصيل" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="مصروفات 2025 - ملخص" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'أوامر الشراء'!$A$1:$L$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'العهد - تفصيل المصروفات'!$A$1:$I$179</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'مصروفات 2025 - تفصيل'!$A$1:$L$307</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'أوامر الشراء'!$A$1:$L$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'العهد - تفصيل المصروفات'!$A$1:$I$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'مصروفات 2025 - تفصيل'!$A$1:$L$307</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -166,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -259,6 +260,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -624,7 +633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -905,6 +914,23 @@
       <c r="A25" s="9" t="inlineStr">
         <is>
           <t>8) مصروفات 2025 مضافة في شيتي "مصروفات 2025 - تفصيل" و"مصروفات 2025 - ملخص".</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="46" t="inlineStr">
+        <is>
+          <t>ثالثاً: مصروفات التشغيل قبل 30-7-2025 (فبراير–ديسمبر 2024)</t>
+        </is>
+      </c>
+      <c r="B27" s="46" t="n"/>
+      <c r="C27" s="47">
+        <f>'مصروفات قبل 30.7.2025'!E28</f>
+        <v/>
+      </c>
+      <c r="D27" s="46" t="inlineStr">
+        <is>
+          <t>تفصيلها في شيت "مصروفات قبل 30.7.2025"</t>
         </is>
       </c>
     </row>
@@ -926,6 +952,685 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="43" t="inlineStr">
+        <is>
+          <t>مصروفات التشغيل – مزرعة الرياض (قبل 30-7-2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="48" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B2" s="48" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="C2" s="48" t="inlineStr">
+        <is>
+          <t>البيان</t>
+        </is>
+      </c>
+      <c r="D2" s="48" t="inlineStr">
+        <is>
+          <t>طريقة الدفع</t>
+        </is>
+      </c>
+      <c r="E2" s="48" t="inlineStr">
+        <is>
+          <t>المبلغ</t>
+        </is>
+      </c>
+      <c r="F2" s="48" t="inlineStr">
+        <is>
+          <t>ملاحظة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="24" t="n">
+        <v>45348</v>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>بيتموس من (شركة المدارات)</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E3" s="25" t="n">
+        <v>4312.5</v>
+      </c>
+      <c r="F3" s="23" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>45399</v>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>حساب إيجار براد في المزرعة</t>
+        </is>
+      </c>
+      <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="24" t="n">
+        <v>45446</v>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>فاتورة كهرباء</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E5" s="25" t="n">
+        <v>1123</v>
+      </c>
+      <c r="F5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>45449</v>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>شجر من جدة</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>30300</v>
+      </c>
+      <c r="F6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="24" t="n">
+        <v>45486</v>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>سماد كمبوست من الصافي</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="24" t="n">
+        <v>45488</v>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>بذور من الواحة</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>51974</v>
+      </c>
+      <c r="F8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="24" t="n">
+        <v>45488</v>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>فاتورة كهرباء</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>555</v>
+      </c>
+      <c r="F9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>45510</v>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>شجر أكاسيا وتبيسيا</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>40000</v>
+      </c>
+      <c r="F10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="24" t="n">
+        <v>45510</v>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>مراكن 35 سم عدد 5000</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>14500</v>
+      </c>
+      <c r="F11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="24" t="n">
+        <v>45510</v>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>مراكن وصواني للزهور من التاج</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E12" s="25" t="n">
+        <v>29038</v>
+      </c>
+      <c r="F12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="24" t="n">
+        <v>45510</v>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>بيتموس وبيرلايت من التكامل</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E13" s="25" t="n">
+        <v>58995</v>
+      </c>
+      <c r="F13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="24" t="n">
+        <v>45510</v>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>فاتورة كهرباء</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E14" s="25" t="n">
+        <v>677</v>
+      </c>
+      <c r="F14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="24" t="n">
+        <v>45511</v>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>مراكن مقاس 12 من أمجاد الخليج</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E15" s="25" t="n">
+        <v>25875</v>
+      </c>
+      <c r="F15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="24" t="n">
+        <v>45547</v>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>كراتين فلين للزهور عدد 5000 كرتونة</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E16" s="25" t="n">
+        <v>11500</v>
+      </c>
+      <c r="F16" s="23" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="24" t="n">
+        <v>45560</v>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>فاتورة كهرباء</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E17" s="25" t="n">
+        <v>928</v>
+      </c>
+      <c r="F17" s="23" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="B18" s="24" t="n">
+        <v>45568</v>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>بيتموس التكامل</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>50715</v>
+      </c>
+      <c r="F18" s="23" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B19" s="24" t="n">
+        <v>45579</v>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>فاتورة كهرباء</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>1775</v>
+      </c>
+      <c r="F19" s="23" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B20" s="24" t="n">
+        <v>45588</v>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>رسوم مكتب الجمرك</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E20" s="25" t="n">
+        <v>3883</v>
+      </c>
+      <c r="F20" s="23" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B21" s="24" t="n">
+        <v>45591</v>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>كراتين فلين للزهور عدد 5000 كرتونة</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E21" s="25" t="n">
+        <v>14375</v>
+      </c>
+      <c r="F21" s="23" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B22" s="24" t="n">
+        <v>45591</v>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>كراتين فلين للزهور عدد 10000 كرتونة</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E22" s="25" t="n">
+        <v>24150</v>
+      </c>
+      <c r="F22" s="23" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="n">
+        <v>23</v>
+      </c>
+      <c r="B23" s="24" t="n">
+        <v>45595</v>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>مراكن 9 سم من التاج</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E23" s="25" t="n">
+        <v>23000</v>
+      </c>
+      <c r="F23" s="23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="36" t="n"/>
+      <c r="B24" s="37" t="n"/>
+      <c r="C24" s="36" t="inlineStr">
+        <is>
+          <t>فاتورة كهرباء</t>
+        </is>
+      </c>
+      <c r="D24" s="36" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E24" s="38" t="n">
+        <v>2043.4</v>
+      </c>
+      <c r="F24" s="36" t="inlineStr">
+        <is>
+          <t>⚠ بدون تاريخ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="36" t="n"/>
+      <c r="B25" s="37" t="n"/>
+      <c r="C25" s="36" t="inlineStr">
+        <is>
+          <t>فاتورة كهرباء</t>
+        </is>
+      </c>
+      <c r="D25" s="36" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E25" s="38" t="n">
+        <v>4886.5</v>
+      </c>
+      <c r="F25" s="36" t="inlineStr">
+        <is>
+          <t>⚠ بدون تاريخ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="36" t="n"/>
+      <c r="B26" s="37" t="n"/>
+      <c r="C26" s="36" t="inlineStr">
+        <is>
+          <t>فاتورة كهرباء</t>
+        </is>
+      </c>
+      <c r="D26" s="36" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E26" s="38" t="n">
+        <v>2716.3</v>
+      </c>
+      <c r="F26" s="36" t="inlineStr">
+        <is>
+          <t>⚠ بدون تاريخ</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="n"/>
+      <c r="B27" s="24" t="n">
+        <v>45636</v>
+      </c>
+      <c r="C27" s="23" t="inlineStr">
+        <is>
+          <t>فاتورة كهرباء</t>
+        </is>
+      </c>
+      <c r="D27" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E27" s="25" t="n">
+        <v>4918.97</v>
+      </c>
+      <c r="F27" s="23" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr"/>
+      <c r="B28" s="21" t="inlineStr"/>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="D28" s="21" t="inlineStr"/>
+      <c r="E28" s="22">
+        <f>SUM(E3:E27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="21" t="n"/>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="49" t="inlineStr"/>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>ملاحظات:</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>1) الإجمالي 412,040.67 مطابق لمجموع البنود.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>2) ⚠ الترقيم ناقص البندين 8 و 17 – يلزم التأكد إن كانا محذوفين أو سقطا من الكشف.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="49" t="inlineStr">
+        <is>
+          <t>3) ⚠ 3 فواتير كهرباء بدون تاريخ (2,043.40 و 4,886.50 و 2,716.30).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>4) ⚠ الكشف يبدأ من 26-2-2024 بينما مبيعات ما قبل الفترة تبدأ من 1-10-2024 – منها 279,577.50 مصروفات قبل 1-10-2024 (فبراير–سبتمبر 2024).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t>5) لا توجد مصروفات مسجلة من 11-12-2024 حتى 30-6-2025 في هذا الكشف (مصروفات 2025 تبدأ من يونيو 2025 في شيت مصروفات 2025).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A29:F29"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2578,7 +3283,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9351,7 +10056,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9786,7 +10491,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24061,7 +24766,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add Riyadh farm establishment expenses sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/المصاريف_التشغيلية_مزرعة_الرياض_2026.xlsx
+++ b/المصاريف_التشغيلية_مزرعة_الرياض_2026.xlsx
@@ -8,17 +8,18 @@
   </bookViews>
   <sheets>
     <sheet name="الملخص" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="مصروفات قبل 30.7.2025" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="أوامر الشراء" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="العهد - تفصيل المصروفات" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="العهد - ملخص" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="مصروفات 2025 - تفصيل" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="مصروفات 2025 - ملخص" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="مصروفات التأسيس" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="مصروفات قبل 30.7.2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="أوامر الشراء" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="العهد - تفصيل المصروفات" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="العهد - ملخص" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="مصروفات 2025 - تفصيل" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="مصروفات 2025 - ملخص" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'أوامر الشراء'!$A$1:$L$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'العهد - تفصيل المصروفات'!$A$1:$I$179</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'مصروفات 2025 - تفصيل'!$A$1:$L$307</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'أوامر الشراء'!$A$1:$L$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'العهد - تفصيل المصروفات'!$A$1:$I$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'مصروفات 2025 - تفصيل'!$A$1:$L$307</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -633,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -931,6 +932,23 @@
       <c r="D27" s="46" t="inlineStr">
         <is>
           <t>تفصيلها في شيت "مصروفات قبل 30.7.2025"</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="46" t="inlineStr">
+        <is>
+          <t>رابعاً: مصروفات التأسيس (صفحة مستقلة)</t>
+        </is>
+      </c>
+      <c r="B28" s="46" t="n"/>
+      <c r="C28" s="47">
+        <f>'مصروفات التأسيس'!E27</f>
+        <v/>
+      </c>
+      <c r="D28" s="46" t="inlineStr">
+        <is>
+          <t>تفصيلها في شيت "مصروفات التأسيس" – غير مجمعة مع المصاريف التشغيلية</t>
         </is>
       </c>
     </row>
@@ -957,6 +975,756 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="43" t="inlineStr">
+        <is>
+          <t>مصروفات تأسيس مزرعة الرياض</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="48" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B2" s="48" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="C2" s="48" t="inlineStr">
+        <is>
+          <t>البيان</t>
+        </is>
+      </c>
+      <c r="D2" s="48" t="inlineStr">
+        <is>
+          <t>طريقة الدفع</t>
+        </is>
+      </c>
+      <c r="E2" s="48" t="inlineStr">
+        <is>
+          <t>المبلغ</t>
+        </is>
+      </c>
+      <c r="F2" s="48" t="inlineStr">
+        <is>
+          <t>ملاحظة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="15" t="n">
+        <v>45292</v>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>مصروفات من حساب الزهور لأبوخالد (عهدة)</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>أبومازن</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="n">
+        <v>88770</v>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>⚠ مدفوع عن طريق أبومازن (ليس من حسابات الشركة) – عهدة بحساب الزهور لأبوخالد</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="15" t="n">
+        <v>45292</v>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>سيارة ونيت غمارتين</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>أبومازن</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>⚠ مدفوع عن طريق أبومازن</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>45300</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>رسوم إيجار لمدة عامين</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>300000</v>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>إيجار سنتين – جزء منه يخص فترة التشغيل (يُراعى عند التحميل)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>45309</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>خلايا تبريد وشبك ظل وبلاستيك بيوت محمية (مصنع الروضة)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>79904</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>45323</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>شراء غطاسات وسيور مراوح (مصنع الروضة)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>6417</v>
+      </c>
+      <c r="F7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>45330</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>شراء شبك ظل (مصنع الروضة)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>7820</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>45335</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>سداد خدمة إيصال التيار الكهربائي ورفعة لقدرة 300 أمبير</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>13330.8</v>
+      </c>
+      <c r="F9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>45348</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>شبك ظل من (شركة فالكون)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>31562</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>45375</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>دفعة أولى من حساب الأسفلت بالمزرعة</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>45375</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>شراء سيارة ايسوزو دينة موديل 2023</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>97750</v>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>45407</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>تأمين السيارات</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>4450</v>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>الترتيب: تاريخه 25-4 قبل بندي 12 و13 بتاريخ 8-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>45390</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>دفعة ثانية من حساب الأسفلت + إيجار شيول 9 أيام</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>11700</v>
+      </c>
+      <c r="F14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>45390</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>بلاستيك أسود تغطية البيوت المحمية (مؤسسة أفكار)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>45403</v>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>سليمان عبدالعزيز الخضيري (توجيه من أبومازن)</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>بنك ساب</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>⚠ دفعة لشخص بتوجيه من أبومازن بدون بيان للغرض</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>45407</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>شراء سيارة ايسوزو غمارتين موديل 2023</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>85400</v>
+      </c>
+      <c r="F17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="12" t="n">
+        <v>45417</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>شراء مضخة (شركة المسبك)</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>5550</v>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>45417</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>شراء شبك ظل (شركة آل طالب)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>31050</v>
+      </c>
+      <c r="F19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="12" t="n">
+        <v>45444</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>صندوق براد للدينة – عصمت</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>14500</v>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>45479</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>كيبل كهرباء (شركة العواد للتجارة)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>8100</v>
+      </c>
+      <c r="F21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>45547</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>حساب غطاس بالمزرعة</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>7300</v>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>45568</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>شراء بيوت جاهزة</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>29900</v>
+      </c>
+      <c r="F23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>45568</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>شراء خزانات مياه</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>29000</v>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>45962</v>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>دينة مندوب الرياض – عماد</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="n">
+        <v>123000</v>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>⚠ التاريخ 1-11-2025 وليس 2024 – خارج فترة التأسيس (يقع ضمن فترة التشغيل)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>45636</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>مواد سباكة من الوسايل</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>36232</v>
+      </c>
+      <c r="F26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr"/>
+      <c r="B27" s="21" t="inlineStr"/>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="D27" s="21" t="inlineStr"/>
+      <c r="E27" s="22">
+        <f>SUM(E3:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="21" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>حسب طريقة الدفع</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="23" t="inlineStr"/>
+      <c r="B30" s="23" t="inlineStr"/>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
+          <t>البنك السعودي</t>
+        </is>
+      </c>
+      <c r="D30" s="23" t="inlineStr"/>
+      <c r="E30" s="25">
+        <f>SUMIFS(E3:E26,D3:D26,C30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="23" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="inlineStr"/>
+      <c r="B31" s="23" t="inlineStr"/>
+      <c r="C31" s="23" t="inlineStr">
+        <is>
+          <t>بنك الرياض</t>
+        </is>
+      </c>
+      <c r="D31" s="23" t="inlineStr"/>
+      <c r="E31" s="25">
+        <f>SUMIFS(E3:E26,D3:D26,C31)</f>
+        <v/>
+      </c>
+      <c r="F31" s="23" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="23" t="inlineStr"/>
+      <c r="B32" s="23" t="inlineStr"/>
+      <c r="C32" s="23" t="inlineStr">
+        <is>
+          <t>بنك ساب</t>
+        </is>
+      </c>
+      <c r="D32" s="23" t="inlineStr"/>
+      <c r="E32" s="25">
+        <f>SUMIFS(E3:E26,D3:D26,C32)</f>
+        <v/>
+      </c>
+      <c r="F32" s="23" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr"/>
+      <c r="B33" s="23" t="inlineStr"/>
+      <c r="C33" s="23" t="inlineStr">
+        <is>
+          <t>أبومازن</t>
+        </is>
+      </c>
+      <c r="D33" s="23" t="inlineStr"/>
+      <c r="E33" s="25">
+        <f>SUMIFS(E3:E26,D3:D26,C33)</f>
+        <v/>
+      </c>
+      <c r="F33" s="23" t="n"/>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="49" t="inlineStr"/>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t>ملاحظات:</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>1) الإجمالي 1,089,735.80 مطابق لمجموع البنود.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="49" t="inlineStr">
+        <is>
+          <t>2) ⚠ البند 23 "دينة مندوب الرياض – عماد" 123,000 تاريخه 1-11-2025 وليس 2024 – يقع داخل فترة التشغيل، يلزم التأكد من التاريخ أو نقله.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="49" t="inlineStr">
+        <is>
+          <t>3) ⚠ البنود 1 و 2 (98,770) مدفوعة عن طريق أبومازن، والبند 14 (35,000) دفعة لسليمان الخضيري بتوجيه منه بدون بيان للغرض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>4) البند 3 إيجار لمدة عامين (300,000) من 9-1-2024 – يغطي حتى يناير 2026 تقريباً، أي أن جزءاً منه يخص فترة التشغيل. وتقرير العهدة 2026 فيه إيجار مزرعة الرياض 150,000 بتاريخ 27-7-2026 (مدفوع من تبوك).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>5) سيارات مشتراة: ايسوزو دينة 97,750 + ايسوزو غمارتين 85,400 + ونيت غمارتين 10,000 + دينة عماد 123,000 + صندوق براد 14,500 + تأمين 4,450.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A39:F39"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1630,7 +2398,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3283,7 +4051,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10056,7 +10824,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10491,7 +11259,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24766,7 +25534,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add expenses paid by Abu Khaled from sales before 30-7-2025
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/المصاريف_التشغيلية_مزرعة_الرياض_2026.xlsx
+++ b/المصاريف_التشغيلية_مزرعة_الرياض_2026.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="yyyy/mm/dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +53,11 @@
     <font>
       <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="9">
@@ -168,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -269,6 +274,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -634,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -650,6 +657,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -918,6 +926,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="46" t="inlineStr">
         <is>
@@ -938,15 +947,32 @@
     <row r="28">
       <c r="A28" s="46" t="inlineStr">
         <is>
-          <t>رابعاً: مصروفات التأسيس (صفحة مستقلة)</t>
+          <t>ثالثاً (ب): مصروفات دفعها م/ عادل أبو خالد من المبيعات (10-2024 إلى 6-2025)</t>
         </is>
       </c>
       <c r="B28" s="46" t="n"/>
       <c r="C28" s="47">
+        <f>'مصروفات قبل 30.7.2025'!E42</f>
+        <v/>
+      </c>
+      <c r="D28" s="46" t="inlineStr">
+        <is>
+          <t>تفصيلها في شيت "مصروفات قبل 30.7.2025"</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="46" t="inlineStr">
+        <is>
+          <t>رابعاً: مصروفات التأسيس (صفحة مستقلة)</t>
+        </is>
+      </c>
+      <c r="B29" s="46" t="n"/>
+      <c r="C29" s="47">
         <f>'مصروفات التأسيس'!E27</f>
         <v/>
       </c>
-      <c r="D28" s="46" t="inlineStr">
+      <c r="D29" s="46" t="inlineStr">
         <is>
           <t>تفصيلها في شيت "مصروفات التأسيس" – غير مجمعة مع المصاريف التشغيلية</t>
         </is>
@@ -1725,7 +1751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2383,10 +2409,157 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="50" t="inlineStr">
+        <is>
+          <t>مصروفات تم دفعها عن طريق م/ عادل أبو خالد (من المبيعات)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="51" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B38" s="51" t="inlineStr">
+        <is>
+          <t>الفترة</t>
+        </is>
+      </c>
+      <c r="C38" s="51" t="inlineStr">
+        <is>
+          <t>البيان</t>
+        </is>
+      </c>
+      <c r="D38" s="51" t="inlineStr">
+        <is>
+          <t>طريقة الدفع</t>
+        </is>
+      </c>
+      <c r="E38" s="51" t="inlineStr">
+        <is>
+          <t>المبلغ</t>
+        </is>
+      </c>
+      <c r="F38" s="51" t="inlineStr">
+        <is>
+          <t>ملاحظة</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B39" s="23" t="inlineStr">
+        <is>
+          <t>10-2024 إلى 12-2024</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="inlineStr">
+        <is>
+          <t>مصروفات دفعت من أبو خالد (من المبيعات)</t>
+        </is>
+      </c>
+      <c r="D39" s="23" t="inlineStr">
+        <is>
+          <t>من المبيعات – م/ عادل</t>
+        </is>
+      </c>
+      <c r="E39" s="25" t="n">
+        <v>122748</v>
+      </c>
+      <c r="F39" s="23" t="inlineStr">
+        <is>
+          <t>إجمالي ربع سنوي بدون تفصيل بنود</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>01-2025 إلى 03-2025</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="inlineStr">
+        <is>
+          <t>مصروفات دفعت من أبو خالد (من المبيعات)</t>
+        </is>
+      </c>
+      <c r="D40" s="23" t="inlineStr">
+        <is>
+          <t>من المبيعات – م/ عادل</t>
+        </is>
+      </c>
+      <c r="E40" s="25" t="n">
+        <v>94298</v>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>إجمالي ربع سنوي بدون تفصيل بنود</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B41" s="23" t="inlineStr">
+        <is>
+          <t>04-2025 إلى 06-2025</t>
+        </is>
+      </c>
+      <c r="C41" s="23" t="inlineStr">
+        <is>
+          <t>مصروفات دفعت من أبو خالد (من المبيعات)</t>
+        </is>
+      </c>
+      <c r="D41" s="23" t="inlineStr">
+        <is>
+          <t>من المبيعات – م/ عادل</t>
+        </is>
+      </c>
+      <c r="E41" s="25" t="n">
+        <v>196190</v>
+      </c>
+      <c r="F41" s="23" t="inlineStr">
+        <is>
+          <t>إجمالي ربع سنوي بدون تفصيل بنود</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="21" t="inlineStr"/>
+      <c r="B42" s="21" t="inlineStr"/>
+      <c r="C42" s="21" t="inlineStr">
+        <is>
+          <t>إجمالي المصروفات المدفوعة عن طريق م/ عادل</t>
+        </is>
+      </c>
+      <c r="D42" s="21" t="inlineStr"/>
+      <c r="E42" s="22">
+        <f>SUM(E39:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="21" t="n"/>
+    </row>
+    <row r="44" ht="48" customHeight="1">
+      <c r="A44" s="49" t="inlineStr">
+        <is>
+          <t>ملاحظات: الإجمالي 413,236.00 مطابق. هذه المصروفات دُفعت من حصيلة المبيعات مباشرة (مبيعات نفس الفترة 610,688.00 بشيت المبيعات) – بدون تفصيل بنود أو مستندات. تغطي الفترة من أكتوبر 2024 إلى يونيو 2025 التي لم يكن بها مصروفات مسجلة بعد 10-12-2024.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
     <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A44:F44"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A37:F37"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A34:F34"/>

</xml_diff>